<commit_message>
Inbetriebnahme v07: Review-Punkt 8 (SPI3-CS Pull-ups) + Firmware-Repo verlinkt
- Review_v07.md: neuer Punkt 8 - je 10 kOhm Pull-up auf 3,3 V am 541-Eingang
  von GPIO18 (MAX7221-CS) und am ungepufferten Netz GPIO15 (MCP23S17-CS);
  ohne sie sind beide CS bis spibus_init() undefiniert, der MAX7221 nimmt
  Stoerflanken als Frame an (Display-Test-Register kam hoch)
- Steuerplatine_Doku.md: Paragraph 11 (Kasten) und 12.14 entsprechend ergaenzt
- Kegelautomat_Steckerbelegung.xlsx aktualisiert
- README.md / CLAUDE.md: Firmware liegt jetzt in bontango/kegelautomat-firmware
  (Stand v0.01), Verweis statt lokalem Pfad
- PROJECT.md und datasheets/Spielregeln.txt neu aufgenommen

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/datasheets/Kegelautomat_Steckerbelegung.xlsx
+++ b/datasheets/Kegelautomat_Steckerbelegung.xlsx
@@ -8,24 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="N:\Projekte\Kegelautomat\datasheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F60FD47-D20F-4D95-AAD8-E91F7065293E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5343B4CB-C53E-4D8D-91D1-1459EDA1D3F3}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
+    <sheet name="Stecker" sheetId="1" r:id="rId1"/>
+    <sheet name="Spielfeld" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">Stecker!$A$1:$AB$68</definedName>
+  </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="157">
   <si>
     <t>J3</t>
   </si>
@@ -304,6 +311,198 @@
   </si>
   <si>
     <t>Power</t>
+  </si>
+  <si>
+    <t>Zahl 1</t>
+  </si>
+  <si>
+    <t>Zahl 9</t>
+  </si>
+  <si>
+    <t>Zahl 8</t>
+  </si>
+  <si>
+    <t>Zahl 7</t>
+  </si>
+  <si>
+    <t>Zahl 6</t>
+  </si>
+  <si>
+    <t>Zahl 5</t>
+  </si>
+  <si>
+    <t>Zahl 4</t>
+  </si>
+  <si>
+    <t>Zahl 3</t>
+  </si>
+  <si>
+    <t>Zahl 2</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>I</t>
+  </si>
+  <si>
+    <t>G</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>T</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>E</t>
+  </si>
+  <si>
+    <t>K</t>
+  </si>
+  <si>
+    <t>Kegel 1</t>
+  </si>
+  <si>
+    <t>Kegel 9</t>
+  </si>
+  <si>
+    <t>Kegel 8</t>
+  </si>
+  <si>
+    <t>Kegel 7</t>
+  </si>
+  <si>
+    <t>Kegel 6</t>
+  </si>
+  <si>
+    <t>Kegel 5</t>
+  </si>
+  <si>
+    <t>Kegel 4</t>
+  </si>
+  <si>
+    <t>Kegel 3</t>
+  </si>
+  <si>
+    <t>Kegel 2</t>
+  </si>
+  <si>
+    <t>Start</t>
+  </si>
+  <si>
+    <t>Münzer NO</t>
+  </si>
+  <si>
+    <t>Münzer NC</t>
+  </si>
+  <si>
+    <t>Kontakt 1</t>
+  </si>
+  <si>
+    <t>Kontakt 3</t>
+  </si>
+  <si>
+    <t>Kontakt 5</t>
+  </si>
+  <si>
+    <t>Kontakt 7</t>
+  </si>
+  <si>
+    <t>Kontakt 9</t>
+  </si>
+  <si>
+    <t>Kontakt 8</t>
+  </si>
+  <si>
+    <t>Kontakt 6</t>
+  </si>
+  <si>
+    <t>Kontakt 4</t>
+  </si>
+  <si>
+    <t>Kontakt 2</t>
+  </si>
+  <si>
+    <t>SLAM Kontakt (NO)</t>
+  </si>
+  <si>
+    <t>Münzannahme</t>
+  </si>
+  <si>
+    <t>Starttaste</t>
+  </si>
+  <si>
+    <t>Ball 1er</t>
+  </si>
+  <si>
+    <t>Ball 10er</t>
+  </si>
+  <si>
+    <t>Credit 1er</t>
+  </si>
+  <si>
+    <t>Credit 10er</t>
+  </si>
+  <si>
+    <t>Score 1er</t>
+  </si>
+  <si>
+    <t>Score 10er</t>
+  </si>
+  <si>
+    <t>Score 100er</t>
+  </si>
+  <si>
+    <t>Score 1000er</t>
+  </si>
+  <si>
+    <t>immer von links nach rechts</t>
+  </si>
+  <si>
+    <t>&lt;=   Kegel 1,3,5,7,9,8,6,4,2</t>
+  </si>
+  <si>
+    <t>&lt;=   B I G S T R I K E</t>
+  </si>
+  <si>
+    <t>&lt;=   Zahl 1,3,5,7,9,8,6,4,2</t>
+  </si>
+  <si>
+    <t>&lt;=   Kontakt 1,3,5,7,9,8,6,4,2</t>
+  </si>
+  <si>
+    <t>Kegel</t>
+  </si>
+  <si>
+    <t>Zahl</t>
+  </si>
+  <si>
+    <t>Kontakt</t>
+  </si>
+  <si>
+    <t>Buchstaben</t>
+  </si>
+  <si>
+    <t>SP1</t>
+  </si>
+  <si>
+    <t>Spule1</t>
+  </si>
+  <si>
+    <t>Münzweiche</t>
+  </si>
+  <si>
+    <t>SP2</t>
+  </si>
+  <si>
+    <t>Spule2</t>
+  </si>
+  <si>
+    <t>Kugelfreigabe</t>
   </si>
 </sst>
 </file>
@@ -327,7 +526,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -358,6 +557,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -371,7 +576,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -379,6 +584,16 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -434,6 +649,109 @@
         <a:xfrm>
           <a:off x="971550" y="7267575"/>
           <a:ext cx="10393225" cy="5601482"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>304800</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>114300</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="1026" name="AutoShape 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{02D38012-69CB-4C65-8978-E16C035F4AF5}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="12192000" y="3048000"/>
+          <a:ext cx="304800" cy="304800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>57150</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>9525</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>698500</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>185738</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Grafik 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F560184-BEE2-43C4-9112-209C42448E98}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4248150" y="200025"/>
+          <a:ext cx="3689350" cy="2767013"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -708,8 +1026,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:S36"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B1:AC36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="27" max="27" width="27.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="2:19" x14ac:dyDescent="0.25">
       <c r="B1" s="3" t="s">
@@ -796,6 +1120,9 @@
       <c r="K3" t="s">
         <v>23</v>
       </c>
+      <c r="L3" t="s">
+        <v>110</v>
+      </c>
       <c r="N3" s="4">
         <v>6</v>
       </c>
@@ -817,6 +1144,9 @@
       <c r="C4" t="s">
         <v>5</v>
       </c>
+      <c r="D4" t="s">
+        <v>93</v>
+      </c>
       <c r="F4" s="4">
         <v>11</v>
       </c>
@@ -830,11 +1160,17 @@
       <c r="K4" t="s">
         <v>24</v>
       </c>
+      <c r="L4" t="s">
+        <v>117</v>
+      </c>
       <c r="N4">
         <v>5</v>
       </c>
       <c r="O4" t="s">
         <v>33</v>
+      </c>
+      <c r="P4" t="s">
+        <v>132</v>
       </c>
       <c r="R4" s="1">
         <v>2</v>
@@ -850,11 +1186,17 @@
       <c r="C5" t="s">
         <v>6</v>
       </c>
+      <c r="D5" t="s">
+        <v>100</v>
+      </c>
       <c r="F5">
         <v>10</v>
       </c>
       <c r="G5" t="s">
         <v>14</v>
+      </c>
+      <c r="H5" t="s">
+        <v>102</v>
       </c>
       <c r="J5" s="4">
         <v>10</v>
@@ -883,17 +1225,26 @@
       <c r="C6" t="s">
         <v>7</v>
       </c>
+      <c r="D6" t="s">
+        <v>98</v>
+      </c>
       <c r="F6">
         <v>9</v>
       </c>
       <c r="G6" t="s">
         <v>15</v>
       </c>
+      <c r="H6" t="s">
+        <v>103</v>
+      </c>
       <c r="J6">
         <v>9</v>
       </c>
       <c r="K6" t="s">
         <v>25</v>
+      </c>
+      <c r="L6" t="s">
+        <v>115</v>
       </c>
       <c r="N6">
         <v>3</v>
@@ -915,23 +1266,35 @@
       <c r="C7" t="s">
         <v>8</v>
       </c>
+      <c r="D7" t="s">
+        <v>96</v>
+      </c>
       <c r="F7">
         <v>8</v>
       </c>
       <c r="G7" t="s">
         <v>16</v>
       </c>
+      <c r="H7" t="s">
+        <v>104</v>
+      </c>
       <c r="J7">
         <v>8</v>
       </c>
       <c r="K7" t="s">
         <v>26</v>
       </c>
+      <c r="L7" t="s">
+        <v>113</v>
+      </c>
       <c r="N7">
         <v>2</v>
       </c>
       <c r="O7" t="s">
         <v>36</v>
+      </c>
+      <c r="P7" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="8" spans="2:19" x14ac:dyDescent="0.25">
@@ -941,17 +1304,26 @@
       <c r="C8" t="s">
         <v>9</v>
       </c>
+      <c r="D8" t="s">
+        <v>94</v>
+      </c>
       <c r="F8">
         <v>7</v>
       </c>
       <c r="G8" t="s">
         <v>17</v>
       </c>
+      <c r="H8" t="s">
+        <v>105</v>
+      </c>
       <c r="J8">
         <v>7</v>
       </c>
       <c r="K8" t="s">
         <v>27</v>
+      </c>
+      <c r="L8" t="s">
+        <v>111</v>
       </c>
       <c r="N8" s="2">
         <v>1</v>
@@ -968,17 +1340,26 @@
       <c r="C9" t="s">
         <v>10</v>
       </c>
+      <c r="D9" t="s">
+        <v>95</v>
+      </c>
       <c r="F9">
         <v>6</v>
       </c>
       <c r="G9" t="s">
         <v>18</v>
       </c>
+      <c r="H9" t="s">
+        <v>106</v>
+      </c>
       <c r="J9">
         <v>6</v>
       </c>
       <c r="K9" t="s">
         <v>28</v>
+      </c>
+      <c r="L9" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="10" spans="2:19" x14ac:dyDescent="0.25">
@@ -988,17 +1369,26 @@
       <c r="C10" t="s">
         <v>11</v>
       </c>
+      <c r="D10" t="s">
+        <v>97</v>
+      </c>
       <c r="F10">
         <v>5</v>
       </c>
       <c r="G10" t="s">
         <v>19</v>
       </c>
+      <c r="H10" t="s">
+        <v>107</v>
+      </c>
       <c r="J10">
         <v>5</v>
       </c>
       <c r="K10" t="s">
         <v>29</v>
+      </c>
+      <c r="L10" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="11" spans="2:19" x14ac:dyDescent="0.25">
@@ -1008,17 +1398,26 @@
       <c r="C11" t="s">
         <v>12</v>
       </c>
+      <c r="D11" t="s">
+        <v>99</v>
+      </c>
       <c r="F11">
         <v>4</v>
       </c>
       <c r="G11" t="s">
         <v>20</v>
       </c>
+      <c r="H11" t="s">
+        <v>103</v>
+      </c>
       <c r="J11">
         <v>4</v>
       </c>
       <c r="K11" t="s">
         <v>30</v>
+      </c>
+      <c r="L11" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="12" spans="2:19" x14ac:dyDescent="0.25">
@@ -1028,17 +1427,35 @@
       <c r="C12" t="s">
         <v>13</v>
       </c>
+      <c r="D12" t="s">
+        <v>101</v>
+      </c>
       <c r="F12">
         <v>3</v>
       </c>
       <c r="G12" t="s">
         <v>21</v>
       </c>
+      <c r="H12" t="s">
+        <v>109</v>
+      </c>
       <c r="J12">
         <v>3</v>
       </c>
       <c r="K12" t="s">
         <v>31</v>
+      </c>
+      <c r="L12" t="s">
+        <v>118</v>
+      </c>
+      <c r="N12" t="s">
+        <v>151</v>
+      </c>
+      <c r="O12" t="s">
+        <v>152</v>
+      </c>
+      <c r="P12" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="13" spans="2:19" x14ac:dyDescent="0.25">
@@ -1055,11 +1472,23 @@
       <c r="G13" t="s">
         <v>22</v>
       </c>
+      <c r="H13" t="s">
+        <v>108</v>
+      </c>
       <c r="J13">
         <v>2</v>
       </c>
       <c r="K13" t="s">
         <v>32</v>
+      </c>
+      <c r="N13" t="s">
+        <v>154</v>
+      </c>
+      <c r="O13" t="s">
+        <v>155</v>
+      </c>
+      <c r="P13" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="14" spans="2:19" x14ac:dyDescent="0.25">
@@ -1085,7 +1514,11 @@
         <v>38</v>
       </c>
     </row>
-    <row r="18" spans="2:17" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:29" x14ac:dyDescent="0.25">
+      <c r="AB17" s="6"/>
+      <c r="AC17" s="6"/>
+    </row>
+    <row r="18" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B18" s="3" t="s">
         <v>0</v>
       </c>
@@ -1098,8 +1531,10 @@
       <c r="O18" s="3" t="s">
         <v>73</v>
       </c>
-    </row>
-    <row r="19" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="AB18" s="6"/>
+      <c r="AC18" s="6"/>
+    </row>
+    <row r="19" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B19" t="s">
         <v>1</v>
       </c>
@@ -1139,8 +1574,10 @@
       <c r="Q19" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="20" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="AB19" s="6"/>
+      <c r="AC19" s="6"/>
+    </row>
+    <row r="20" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B20">
         <v>12</v>
       </c>
@@ -1150,12 +1587,18 @@
       <c r="D20" t="s">
         <v>45</v>
       </c>
+      <c r="E20" t="s">
+        <v>122</v>
+      </c>
       <c r="G20">
         <v>6</v>
       </c>
       <c r="H20" t="s">
         <v>63</v>
       </c>
+      <c r="J20" t="s">
+        <v>119</v>
+      </c>
       <c r="M20" s="1" t="s">
         <v>71</v>
       </c>
@@ -1168,8 +1611,13 @@
       <c r="P20" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="21" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q20" t="s">
+        <v>134</v>
+      </c>
+      <c r="AB20" s="6"/>
+      <c r="AC20" s="6"/>
+    </row>
+    <row r="21" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B21">
         <v>11</v>
       </c>
@@ -1178,6 +1626,9 @@
       </c>
       <c r="D21" t="s">
         <v>46</v>
+      </c>
+      <c r="E21" t="s">
+        <v>123</v>
       </c>
       <c r="G21" s="4">
         <v>5</v>
@@ -1199,8 +1650,13 @@
       <c r="P21" t="s">
         <v>76</v>
       </c>
-    </row>
-    <row r="22" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q21" t="s">
+        <v>135</v>
+      </c>
+      <c r="AB21" s="6"/>
+      <c r="AC21" s="6"/>
+    </row>
+    <row r="22" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B22">
         <v>10</v>
       </c>
@@ -1210,12 +1666,18 @@
       <c r="D22" t="s">
         <v>47</v>
       </c>
+      <c r="E22" t="s">
+        <v>124</v>
+      </c>
       <c r="G22">
         <v>4</v>
       </c>
       <c r="H22" t="s">
         <v>64</v>
       </c>
+      <c r="J22" t="s">
+        <v>120</v>
+      </c>
       <c r="M22" s="1" t="s">
         <v>71</v>
       </c>
@@ -1228,8 +1690,13 @@
       <c r="P22" t="s">
         <v>77</v>
       </c>
-    </row>
-    <row r="23" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q22" t="s">
+        <v>136</v>
+      </c>
+      <c r="AB22" s="6"/>
+      <c r="AC22" s="6"/>
+    </row>
+    <row r="23" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B23">
         <v>9</v>
       </c>
@@ -1239,12 +1706,18 @@
       <c r="D23" t="s">
         <v>48</v>
       </c>
+      <c r="E23" t="s">
+        <v>125</v>
+      </c>
       <c r="G23">
         <v>3</v>
       </c>
       <c r="H23" t="s">
         <v>65</v>
       </c>
+      <c r="J23" t="s">
+        <v>121</v>
+      </c>
       <c r="M23" s="1" t="s">
         <v>71</v>
       </c>
@@ -1257,8 +1730,13 @@
       <c r="P23" t="s">
         <v>75</v>
       </c>
-    </row>
-    <row r="24" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q23" t="s">
+        <v>137</v>
+      </c>
+      <c r="AB23" s="6"/>
+      <c r="AC23" s="6"/>
+    </row>
+    <row r="24" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B24">
         <v>8</v>
       </c>
@@ -1268,12 +1746,18 @@
       <c r="D24" t="s">
         <v>49</v>
       </c>
+      <c r="E24" t="s">
+        <v>126</v>
+      </c>
       <c r="G24">
         <v>2</v>
       </c>
       <c r="H24" t="s">
         <v>66</v>
       </c>
+      <c r="J24" t="s">
+        <v>131</v>
+      </c>
       <c r="M24" s="1" t="s">
         <v>71</v>
       </c>
@@ -1286,8 +1770,13 @@
       <c r="P24" t="s">
         <v>78</v>
       </c>
-    </row>
-    <row r="25" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q24" t="s">
+        <v>138</v>
+      </c>
+      <c r="AB24" s="6"/>
+      <c r="AC24" s="6"/>
+    </row>
+    <row r="25" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B25">
         <v>7</v>
       </c>
@@ -1296,6 +1785,9 @@
       </c>
       <c r="D25" t="s">
         <v>50</v>
+      </c>
+      <c r="E25" t="s">
+        <v>127</v>
       </c>
       <c r="G25" s="1">
         <v>1</v>
@@ -1317,8 +1809,13 @@
       <c r="P25" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="26" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q25" t="s">
+        <v>139</v>
+      </c>
+      <c r="AB25" s="6"/>
+      <c r="AC25" s="6"/>
+    </row>
+    <row r="26" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B26">
         <v>6</v>
       </c>
@@ -1328,6 +1825,9 @@
       <c r="D26" t="s">
         <v>51</v>
       </c>
+      <c r="E26" t="s">
+        <v>128</v>
+      </c>
       <c r="M26" s="1" t="s">
         <v>71</v>
       </c>
@@ -1340,8 +1840,13 @@
       <c r="P26" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="27" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q26" t="s">
+        <v>140</v>
+      </c>
+      <c r="AB26" s="6"/>
+      <c r="AC26" s="6"/>
+    </row>
+    <row r="27" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B27">
         <v>5</v>
       </c>
@@ -1366,8 +1871,13 @@
       <c r="P27" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="28" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q27" t="s">
+        <v>141</v>
+      </c>
+      <c r="AB27" s="6"/>
+      <c r="AC27" s="6"/>
+    </row>
+    <row r="28" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B28">
         <v>4</v>
       </c>
@@ -1377,6 +1887,9 @@
       <c r="D28" t="s">
         <v>68</v>
       </c>
+      <c r="E28" t="s">
+        <v>129</v>
+      </c>
       <c r="M28" s="5" t="s">
         <v>37</v>
       </c>
@@ -1389,8 +1902,10 @@
       <c r="P28" s="5" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="29" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="AB28" s="6"/>
+      <c r="AC28" s="6"/>
+    </row>
+    <row r="29" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B29">
         <v>3</v>
       </c>
@@ -1400,6 +1915,9 @@
       <c r="D29" t="s">
         <v>69</v>
       </c>
+      <c r="E29" t="s">
+        <v>130</v>
+      </c>
       <c r="M29" s="6" t="s">
         <v>82</v>
       </c>
@@ -1412,8 +1930,13 @@
       <c r="P29" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="30" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q29" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="AB29" s="6"/>
+      <c r="AC29" s="6"/>
+    </row>
+    <row r="30" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B30" s="4">
         <v>2</v>
       </c>
@@ -1434,8 +1957,11 @@
       <c r="P30" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="31" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q30" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="31" spans="2:29" x14ac:dyDescent="0.25">
       <c r="B31" s="1">
         <v>1</v>
       </c>
@@ -1456,8 +1982,11 @@
       <c r="P31" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="32" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="Q31" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="32" spans="2:29" x14ac:dyDescent="0.25">
       <c r="M32" t="s">
         <v>85</v>
       </c>
@@ -1470,8 +1999,11 @@
       <c r="P32" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="33" spans="13:16" x14ac:dyDescent="0.25">
+      <c r="Q32" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="33" spans="13:17" x14ac:dyDescent="0.25">
       <c r="M33" t="s">
         <v>86</v>
       </c>
@@ -1484,8 +2016,11 @@
       <c r="P33" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="34" spans="13:16" x14ac:dyDescent="0.25">
+      <c r="Q33" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="34" spans="13:17" x14ac:dyDescent="0.25">
       <c r="M34" t="s">
         <v>87</v>
       </c>
@@ -1498,8 +2033,11 @@
       <c r="P34" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="35" spans="13:16" x14ac:dyDescent="0.25">
+      <c r="Q34" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="35" spans="13:17" x14ac:dyDescent="0.25">
       <c r="M35" t="s">
         <v>88</v>
       </c>
@@ -1512,8 +2050,11 @@
       <c r="P35" s="1" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="36" spans="13:16" x14ac:dyDescent="0.25">
+      <c r="Q35" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="36" spans="13:17" x14ac:dyDescent="0.25">
       <c r="M36" t="s">
         <v>89</v>
       </c>
@@ -1526,9 +2067,211 @@
       <c r="P36" s="1" t="s">
         <v>71</v>
       </c>
+      <c r="Q36" t="s">
+        <v>89</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="8" scale="70" orientation="landscape" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{736B2C48-96D1-45B4-BFBF-0C9B0BC16E5A}">
+  <dimension ref="A1:P15"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="10" width="5.7109375" customWidth="1"/>
+    <col min="16" max="16" width="25.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A1" s="8"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
+      <c r="I1" s="8"/>
+      <c r="J1" s="8"/>
+    </row>
+    <row r="2" spans="1:16" ht="54" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="B2" s="8">
+        <v>1</v>
+      </c>
+      <c r="C2" s="8">
+        <v>3</v>
+      </c>
+      <c r="D2" s="8">
+        <v>5</v>
+      </c>
+      <c r="E2" s="8">
+        <v>7</v>
+      </c>
+      <c r="F2" s="8">
+        <v>9</v>
+      </c>
+      <c r="G2" s="8">
+        <v>8</v>
+      </c>
+      <c r="H2" s="8">
+        <v>6</v>
+      </c>
+      <c r="I2" s="8">
+        <v>4</v>
+      </c>
+      <c r="J2" s="8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A3" s="10" t="s">
+        <v>150</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>107</v>
+      </c>
+      <c r="H3" s="9" t="s">
+        <v>103</v>
+      </c>
+      <c r="I3" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="J3" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="P3" s="7"/>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A4" s="10" t="s">
+        <v>148</v>
+      </c>
+      <c r="B4" s="9">
+        <v>1</v>
+      </c>
+      <c r="C4" s="9">
+        <v>3</v>
+      </c>
+      <c r="D4" s="9">
+        <v>5</v>
+      </c>
+      <c r="E4" s="9">
+        <v>7</v>
+      </c>
+      <c r="F4" s="9">
+        <v>9</v>
+      </c>
+      <c r="G4" s="9">
+        <v>8</v>
+      </c>
+      <c r="H4" s="9">
+        <v>6</v>
+      </c>
+      <c r="I4" s="9">
+        <v>4</v>
+      </c>
+      <c r="J4" s="9">
+        <v>2</v>
+      </c>
+      <c r="P4" s="7" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A5" s="10" t="s">
+        <v>149</v>
+      </c>
+      <c r="B5" s="9">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9">
+        <v>3</v>
+      </c>
+      <c r="D5" s="9">
+        <v>5</v>
+      </c>
+      <c r="E5" s="9">
+        <v>7</v>
+      </c>
+      <c r="F5" s="9">
+        <v>9</v>
+      </c>
+      <c r="G5" s="9">
+        <v>8</v>
+      </c>
+      <c r="H5" s="9">
+        <v>6</v>
+      </c>
+      <c r="I5" s="9">
+        <v>4</v>
+      </c>
+      <c r="J5" s="9">
+        <v>2</v>
+      </c>
+      <c r="P5" s="7"/>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P6" s="7"/>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P7" s="7" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P8" s="7"/>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P9" s="7" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P10" s="7"/>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P11" s="7"/>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P12" s="7"/>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P13" s="7" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P14" s="7"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="P15" s="7" t="s">
+        <v>142</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
 </worksheet>

</xml_diff>